<commit_message>
Should be final and ready to run
</commit_message>
<xml_diff>
--- a/reminder_messages.xlsx
+++ b/reminder_messages.xlsx
@@ -551,7 +551,7 @@
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t xml:space="preserve">0215241 bị sai số điện thoại; Đã gửi tin nhắn; </t>
+          <t xml:space="preserve">Số điện thoại 0215241 bị sai; Đã gửi tin nhắn cho 0912175971; </t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
@@ -620,7 +620,7 @@
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t xml:space="preserve">0 bị sai số điện thoại; Đã gửi tin nhắn; </t>
+          <t xml:space="preserve">Đã gửi tin nhắn cho 0837893181; </t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
@@ -689,7 +689,7 @@
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t xml:space="preserve">0 bị sai số điện thoại; Đã gửi tin nhắn; </t>
+          <t xml:space="preserve">Đã gửi tin nhắn cho 0906150357; </t>
         </is>
       </c>
       <c r="M4" t="inlineStr"/>
@@ -758,7 +758,7 @@
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t xml:space="preserve">037394864 bị sai số điện thoại; 0 bị sai số điện thoại; </t>
+          <t xml:space="preserve">Số điện thoại 037394864 bị sai; </t>
         </is>
       </c>
       <c r="M5" t="inlineStr">
@@ -827,7 +827,7 @@
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t xml:space="preserve">0 bị sai số điện thoại; Đã gửi tin nhắn; </t>
+          <t xml:space="preserve">Đã gửi tin nhắn cho 0972097519; </t>
         </is>
       </c>
       <c r="M6" t="inlineStr">
@@ -896,7 +896,7 @@
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t xml:space="preserve">Đã gửi tin nhắn; Đã gửi tin nhắn; </t>
+          <t xml:space="preserve">Đã gửi tin nhắn cho 0988667651; Đã gửi tin nhắn cho 0985930016; </t>
         </is>
       </c>
       <c r="M7" t="inlineStr"/>
@@ -965,7 +965,7 @@
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t xml:space="preserve">0 bị sai số điện thoại; Đã gửi tin nhắn; </t>
+          <t xml:space="preserve">Đã gửi tin nhắn cho 0342086382; </t>
         </is>
       </c>
       <c r="M8" t="inlineStr">
@@ -1034,7 +1034,7 @@
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t xml:space="preserve">0 bị sai số điện thoại; Đã gửi tin nhắn; </t>
+          <t xml:space="preserve">Đã gửi tin nhắn cho 0912442775; </t>
         </is>
       </c>
       <c r="M9" t="inlineStr">
@@ -1103,7 +1103,7 @@
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t xml:space="preserve">0 bị sai số điện thoại; 0943227890 không dùng Zalo; </t>
+          <t xml:space="preserve">0943227890 không dùng Zalo; </t>
         </is>
       </c>
       <c r="M10" t="inlineStr"/>
@@ -1168,7 +1168,7 @@
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t xml:space="preserve">0 bị sai số điện thoại; Đã gửi tin nhắn; </t>
+          <t xml:space="preserve">Đã gửi tin nhắn cho 0905061978; </t>
         </is>
       </c>
       <c r="M11" t="inlineStr"/>
@@ -1237,7 +1237,7 @@
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t xml:space="preserve">0 bị sai số điện thoại; Đã gửi tin nhắn; </t>
+          <t xml:space="preserve">Đã gửi tin nhắn cho 0968419933; </t>
         </is>
       </c>
       <c r="M12" t="inlineStr">
@@ -1306,7 +1306,7 @@
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t xml:space="preserve">0 bị sai số điện thoại; Đã gửi tin nhắn; </t>
+          <t xml:space="preserve">Đã gửi tin nhắn cho 0978485131; </t>
         </is>
       </c>
       <c r="M13" t="inlineStr">
@@ -1375,7 +1375,7 @@
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t xml:space="preserve">0 bị sai số điện thoại; 0902249935 không dùng Zalo; </t>
+          <t xml:space="preserve">0902249935 không dùng Zalo; </t>
         </is>
       </c>
       <c r="M14" t="inlineStr"/>
@@ -1440,7 +1440,7 @@
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t xml:space="preserve">Đã gửi tin nhắn; Đã gửi tin nhắn; </t>
+          <t xml:space="preserve">Đã gửi tin nhắn cho 0398467174; Đã gửi tin nhắn cho 0965225672; </t>
         </is>
       </c>
       <c r="M15" t="inlineStr">

</xml_diff>